<commit_message>
walk through single-feature classification at all three levels for every grouping
</commit_message>
<xml_diff>
--- a/03_Group_comparisons/HRvLR/05_Classification/03_Modules/c_data/module_classification.xlsx
+++ b/03_Group_comparisons/HRvLR/05_Classification/03_Modules/c_data/module_classification.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="246">
   <si>
     <t>sheet</t>
   </si>
@@ -307,10 +307,10 @@
     <t>design</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/01_Design_Contrasts/c_data/design.rds</t>
-  </si>
-  <si>
-    <t>96d863835b9c36a26e09b4706fc4e5e6</t>
+    <t>03_Group_comparisons/HRvLR/01_Design_Contrasts/c_data/design.rds</t>
+  </si>
+  <si>
+    <t>2eec838bcc442e8a2ff1534078b14a38</t>
   </si>
   <si>
     <t>modules</t>
@@ -418,12 +418,33 @@
     <t>1.2.1</t>
   </si>
   <si>
+    <t>enrichVolcano</t>
+  </si>
+  <si>
+    <t>0.3.0.9000</t>
+  </si>
+  <si>
+    <t>Github (Dustyn-T-Lewis/enrichVolcano@d3fed631f4ae95e01bd61137699313f8de5cc86e)</t>
+  </si>
+  <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
     <t>foreach</t>
   </si>
   <si>
@@ -475,6 +496,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -487,12 +520,27 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
+    <t>labeling</t>
+  </si>
+  <si>
+    <t>0.4.3</t>
+  </si>
+  <si>
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>magrittr</t>
   </si>
   <si>
@@ -505,6 +553,12 @@
     <t>1.5.0</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -517,6 +571,12 @@
     <t>2.0.3</t>
   </si>
   <si>
+    <t>plyr</t>
+  </si>
+  <si>
+    <t>1.8.9</t>
+  </si>
+  <si>
     <t>png</t>
   </si>
   <si>
@@ -538,6 +598,9 @@
     <t>1.2.2</t>
   </si>
   <si>
+    <t>2.44.0</t>
+  </si>
+  <si>
     <t>R6</t>
   </si>
   <si>
@@ -568,6 +631,12 @@
     <t>1.2.3</t>
   </si>
   <si>
+    <t>reshape2</t>
+  </si>
+  <si>
+    <t>1.4.5</t>
+  </si>
+  <si>
     <t>rjson</t>
   </si>
   <si>
@@ -580,6 +649,12 @@
     <t>1.3.0</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -665,6 +740,24 @@
   </si>
   <si>
     <t>3.0.2</t>
+  </si>
+  <si>
+    <t>writexl</t>
+  </si>
+  <si>
+    <t>2.0.1</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -4608,7 +4701,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -4795,15 +4888,15 @@
         <v>133</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C18" t="s">
         <v>105</v>
@@ -4811,10 +4904,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B19" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C19" t="s">
         <v>105</v>
@@ -4822,10 +4915,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B20" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C20" t="s">
         <v>105</v>
@@ -4833,10 +4926,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B21" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C21" t="s">
         <v>105</v>
@@ -4844,10 +4937,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B22" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C22" t="s">
         <v>105</v>
@@ -4855,10 +4948,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B23" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C23" t="s">
         <v>105</v>
@@ -4866,10 +4959,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B24" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C24" t="s">
         <v>105</v>
@@ -4877,10 +4970,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C25" t="s">
         <v>105</v>
@@ -4888,10 +4981,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C26" t="s">
         <v>105</v>
@@ -4899,21 +4992,21 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C27" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B28" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C28" t="s">
         <v>105</v>
@@ -4921,10 +5014,10 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B29" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C29" t="s">
         <v>105</v>
@@ -4932,10 +5025,10 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B30" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C30" t="s">
         <v>105</v>
@@ -4943,10 +5036,10 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B31" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C31" t="s">
         <v>105</v>
@@ -4954,21 +5047,21 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B32" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C32" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C33" t="s">
         <v>105</v>
@@ -4976,10 +5069,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B34" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C34" t="s">
         <v>105</v>
@@ -4987,13 +5080,13 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C35" t="s">
-        <v>169</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -5012,7 +5105,7 @@
         <v>172</v>
       </c>
       <c r="B37" t="s">
-        <v>173</v>
+        <v>136</v>
       </c>
       <c r="C37" t="s">
         <v>105</v>
@@ -5020,10 +5113,10 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>173</v>
+      </c>
+      <c r="B38" t="s">
         <v>174</v>
-      </c>
-      <c r="B38" t="s">
-        <v>175</v>
       </c>
       <c r="C38" t="s">
         <v>105</v>
@@ -5031,10 +5124,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>175</v>
+      </c>
+      <c r="B39" t="s">
         <v>176</v>
-      </c>
-      <c r="B39" t="s">
-        <v>177</v>
       </c>
       <c r="C39" t="s">
         <v>105</v>
@@ -5042,10 +5135,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>177</v>
+      </c>
+      <c r="B40" t="s">
         <v>178</v>
-      </c>
-      <c r="B40" t="s">
-        <v>179</v>
       </c>
       <c r="C40" t="s">
         <v>105</v>
@@ -5053,10 +5146,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>179</v>
+      </c>
+      <c r="B41" t="s">
         <v>180</v>
-      </c>
-      <c r="B41" t="s">
-        <v>181</v>
       </c>
       <c r="C41" t="s">
         <v>105</v>
@@ -5064,10 +5157,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>181</v>
+      </c>
+      <c r="B42" t="s">
         <v>182</v>
-      </c>
-      <c r="B42" t="s">
-        <v>183</v>
       </c>
       <c r="C42" t="s">
         <v>105</v>
@@ -5075,21 +5168,21 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
+        <v>183</v>
+      </c>
+      <c r="B43" t="s">
         <v>184</v>
       </c>
-      <c r="B43" t="s">
-        <v>185</v>
-      </c>
       <c r="C43" t="s">
-        <v>169</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
+        <v>185</v>
+      </c>
+      <c r="B44" t="s">
         <v>186</v>
-      </c>
-      <c r="B44" t="s">
-        <v>187</v>
       </c>
       <c r="C44" t="s">
         <v>105</v>
@@ -5097,13 +5190,13 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
+        <v>187</v>
+      </c>
+      <c r="B45" t="s">
         <v>188</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>189</v>
-      </c>
-      <c r="C45" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -5119,21 +5212,21 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" t="s">
         <v>192</v>
       </c>
-      <c r="B47" t="s">
-        <v>193</v>
-      </c>
       <c r="C47" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
+        <v>193</v>
+      </c>
+      <c r="B48" t="s">
         <v>194</v>
-      </c>
-      <c r="B48" t="s">
-        <v>195</v>
       </c>
       <c r="C48" t="s">
         <v>105</v>
@@ -5141,10 +5234,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
+        <v>195</v>
+      </c>
+      <c r="B49" t="s">
         <v>196</v>
-      </c>
-      <c r="B49" t="s">
-        <v>197</v>
       </c>
       <c r="C49" t="s">
         <v>105</v>
@@ -5152,10 +5245,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
+        <v>197</v>
+      </c>
+      <c r="B50" t="s">
         <v>198</v>
-      </c>
-      <c r="B50" t="s">
-        <v>199</v>
       </c>
       <c r="C50" t="s">
         <v>105</v>
@@ -5163,10 +5256,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
+        <v>199</v>
+      </c>
+      <c r="B51" t="s">
         <v>200</v>
-      </c>
-      <c r="B51" t="s">
-        <v>201</v>
       </c>
       <c r="C51" t="s">
         <v>105</v>
@@ -5174,10 +5267,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>201</v>
+      </c>
+      <c r="B52" t="s">
         <v>202</v>
-      </c>
-      <c r="B52" t="s">
-        <v>203</v>
       </c>
       <c r="C52" t="s">
         <v>105</v>
@@ -5185,10 +5278,10 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>203</v>
+      </c>
+      <c r="B53" t="s">
         <v>204</v>
-      </c>
-      <c r="B53" t="s">
-        <v>205</v>
       </c>
       <c r="C53" t="s">
         <v>105</v>
@@ -5196,10 +5289,10 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>205</v>
+      </c>
+      <c r="B54" t="s">
         <v>206</v>
-      </c>
-      <c r="B54" t="s">
-        <v>131</v>
       </c>
       <c r="C54" t="s">
         <v>105</v>
@@ -5213,7 +5306,7 @@
         <v>208</v>
       </c>
       <c r="C55" t="s">
-        <v>105</v>
+        <v>189</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -5246,6 +5339,182 @@
         <v>214</v>
       </c>
       <c r="C58" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>215</v>
+      </c>
+      <c r="B59" t="s">
+        <v>216</v>
+      </c>
+      <c r="C59" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" t="s">
+        <v>217</v>
+      </c>
+      <c r="B60" t="s">
+        <v>218</v>
+      </c>
+      <c r="C60" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>219</v>
+      </c>
+      <c r="B61" t="s">
+        <v>220</v>
+      </c>
+      <c r="C61" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" t="s">
+        <v>221</v>
+      </c>
+      <c r="B62" t="s">
+        <v>222</v>
+      </c>
+      <c r="C62" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" t="s">
+        <v>223</v>
+      </c>
+      <c r="B63" t="s">
+        <v>224</v>
+      </c>
+      <c r="C63" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" t="s">
+        <v>225</v>
+      </c>
+      <c r="B64" t="s">
+        <v>226</v>
+      </c>
+      <c r="C64" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>227</v>
+      </c>
+      <c r="B65" t="s">
+        <v>228</v>
+      </c>
+      <c r="C65" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>229</v>
+      </c>
+      <c r="B66" t="s">
+        <v>230</v>
+      </c>
+      <c r="C66" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>231</v>
+      </c>
+      <c r="B67" t="s">
+        <v>131</v>
+      </c>
+      <c r="C67" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
+        <v>232</v>
+      </c>
+      <c r="B68" t="s">
+        <v>233</v>
+      </c>
+      <c r="C68" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>234</v>
+      </c>
+      <c r="B69" t="s">
+        <v>235</v>
+      </c>
+      <c r="C69" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
+        <v>236</v>
+      </c>
+      <c r="B70" t="s">
+        <v>237</v>
+      </c>
+      <c r="C70" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>238</v>
+      </c>
+      <c r="B71" t="s">
+        <v>239</v>
+      </c>
+      <c r="C71" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
+        <v>240</v>
+      </c>
+      <c r="B72" t="s">
+        <v>241</v>
+      </c>
+      <c r="C72" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>242</v>
+      </c>
+      <c r="B73" t="s">
+        <v>243</v>
+      </c>
+      <c r="C73" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
+        <v>244</v>
+      </c>
+      <c r="B74" t="s">
+        <v>245</v>
+      </c>
+      <c r="C74" t="s">
         <v>105</v>
       </c>
     </row>

</xml_diff>